<commit_message>
data: refresh leaderboard (2026-08-27)
</commit_message>
<xml_diff>
--- a/public/downloads/AlonsoStrain2023.xlsx
+++ b/public/downloads/AlonsoStrain2023.xlsx
@@ -1557,16 +1557,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>0.003619283792173898</v>
+        <v>0.00570079489939479</v>
       </c>
       <c r="O3" s="5">
         <v>906</v>
       </c>
       <c r="P3" s="4">
-        <v>0.09279800302524552</v>
+        <v>0.09279170024202681</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.08658571366901505</v>
+        <v>0.08655858753214007</v>
       </c>
       <c r="R3" s="5">
         <v>906</v>
@@ -1616,16 +1616,16 @@
         <v>58</v>
       </c>
       <c r="N4" s="4">
-        <v>0.9375551521379093</v>
+        <v>0.59701191433048</v>
       </c>
       <c r="O4" s="5">
         <v>733</v>
       </c>
       <c r="P4" s="4">
-        <v>1.651154583878645</v>
+        <v>1.568472535920416</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.3719211319241655</v>
+        <v>0.1869449797720189</v>
       </c>
       <c r="R4" s="5">
         <v>685</v>
@@ -1675,22 +1675,22 @@
         <v>48</v>
       </c>
       <c r="N5" s="4">
-        <v>0.3238937692369147</v>
+        <v>0.01217034946572593</v>
       </c>
       <c r="O5" s="5">
         <v>635</v>
       </c>
       <c r="P5" s="4">
-        <v>1.393499329906395</v>
+        <v>1.28225661489716</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.3585449647558011</v>
+        <v>0.1315097870805919</v>
       </c>
       <c r="R5" s="5">
-        <v>591</v>
+        <v>587</v>
       </c>
       <c r="S5" s="5">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1857,16 +1857,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>-0.2044059334387915</v>
+        <v>-0.1874583699172945</v>
       </c>
       <c r="O3" s="5">
         <v>851</v>
       </c>
       <c r="P3" s="4">
-        <v>0.2016688685529673</v>
+        <v>0.2016719101679769</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.1903024239249593</v>
+        <v>0.1896329352947825</v>
       </c>
       <c r="R3" s="5">
         <v>851</v>
@@ -1916,22 +1916,22 @@
         <v>101</v>
       </c>
       <c r="N4" s="4">
-        <v>1.247397173131994</v>
+        <v>0.8415630475965372</v>
       </c>
       <c r="O4" s="5">
         <v>686</v>
       </c>
       <c r="P4" s="4">
-        <v>1.015137207472956</v>
+        <v>0.9619988406016615</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.5704116245415298</v>
+        <v>0.3994373945384755</v>
       </c>
       <c r="R4" s="5">
-        <v>627</v>
+        <v>623</v>
       </c>
       <c r="S4" s="5">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="25" customHeight="1">
@@ -1975,22 +1975,22 @@
         <v>32</v>
       </c>
       <c r="N5" s="4">
-        <v>0.3666159674361618</v>
+        <v>0.1802942541226003</v>
       </c>
       <c r="O5" s="5">
         <v>550</v>
       </c>
       <c r="P5" s="4">
-        <v>0.7283401058271604</v>
+        <v>0.7127121344550674</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.4019104994035934</v>
+        <v>0.3595983597974263</v>
       </c>
       <c r="R5" s="5">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="S5" s="5">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -2157,16 +2157,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>0.06758711403143478</v>
+        <v>0.06391484473433628</v>
       </c>
       <c r="O3" s="5">
         <v>863</v>
       </c>
       <c r="P3" s="4">
-        <v>0.1070681769080011</v>
+        <v>0.1070902825328268</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.09375849520376456</v>
+        <v>0.09372266686547262</v>
       </c>
       <c r="R3" s="5">
         <v>863</v>
@@ -2216,16 +2216,16 @@
         <v>0</v>
       </c>
       <c r="N4" s="4">
-        <v>0.5288203692683235</v>
+        <v>0.5326159710056331</v>
       </c>
       <c r="O4" s="5">
         <v>825</v>
       </c>
       <c r="P4" s="4">
-        <v>0.1820652230963759</v>
+        <v>0.1820659370491772</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.1575525373591131</v>
+        <v>0.1575165043239048</v>
       </c>
       <c r="R4" s="5">
         <v>825</v>
@@ -2275,16 +2275,16 @@
         <v>7</v>
       </c>
       <c r="N5" s="4">
-        <v>-0.04447902433617364</v>
+        <v>0.03582684817150206</v>
       </c>
       <c r="O5" s="5">
         <v>740</v>
       </c>
       <c r="P5" s="4">
-        <v>0.2777432615016237</v>
+        <v>0.2611632127829631</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.1765125731106132</v>
+        <v>0.1567509029282786</v>
       </c>
       <c r="R5" s="5">
         <v>733</v>
@@ -2457,16 +2457,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>-0.09461727144166959</v>
+        <v>-0.08912574901751213</v>
       </c>
       <c r="O3" s="5">
         <v>874</v>
       </c>
       <c r="P3" s="4">
-        <v>0.2151007541900198</v>
+        <v>0.2153281437875934</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.1987831788120364</v>
+        <v>0.1987371975015834</v>
       </c>
       <c r="R3" s="5">
         <v>874</v>
@@ -2516,16 +2516,16 @@
         <v>21</v>
       </c>
       <c r="N4" s="4">
-        <v>1.013791610127357</v>
+        <v>0.6774671002563082</v>
       </c>
       <c r="O4" s="5">
         <v>684</v>
       </c>
       <c r="P4" s="4">
-        <v>3.799907251233735</v>
+        <v>3.784030361881833</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.4048345501024522</v>
+        <v>0.2986248647518581</v>
       </c>
       <c r="R4" s="5">
         <v>664</v>
@@ -2575,22 +2575,22 @@
         <v>34</v>
       </c>
       <c r="N5" s="4">
-        <v>0.9292749066123122</v>
+        <v>0.07646265750736347</v>
       </c>
       <c r="O5" s="5">
         <v>604</v>
       </c>
       <c r="P5" s="4">
-        <v>3.178314805562774</v>
+        <v>2.881157085132974</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.8574251799673623</v>
+        <v>0.261336835876603</v>
       </c>
       <c r="R5" s="5">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="S5" s="5">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2757,16 +2757,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>0.002275395919727423</v>
+        <v>0.003864530805003596</v>
       </c>
       <c r="O3" s="5">
         <v>902</v>
       </c>
       <c r="P3" s="4">
-        <v>0.0912091126130779</v>
+        <v>0.09121385940047234</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.08412537067882105</v>
+        <v>0.08411086933533615</v>
       </c>
       <c r="R3" s="5">
         <v>902</v>
@@ -2816,22 +2816,22 @@
         <v>112</v>
       </c>
       <c r="N4" s="4">
-        <v>2.080453739519645</v>
+        <v>0.6864566326257773</v>
       </c>
       <c r="O4" s="5">
         <v>773</v>
       </c>
       <c r="P4" s="4">
-        <v>2.871590120617022</v>
+        <v>2.1679284959472</v>
       </c>
       <c r="Q4" s="4">
-        <v>1.410890037703731</v>
+        <v>0.1399944082200012</v>
       </c>
       <c r="R4" s="5">
-        <v>670</v>
+        <v>661</v>
       </c>
       <c r="S4" s="5">
-        <v>103</v>
+        <v>112</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="25" customHeight="1">
@@ -2875,22 +2875,22 @@
         <v>94</v>
       </c>
       <c r="N5" s="4">
-        <v>1.32523703366444</v>
+        <v>0.006423902734240983</v>
       </c>
       <c r="O5" s="5">
         <v>659</v>
       </c>
       <c r="P5" s="4">
-        <v>2.701321121786875</v>
+        <v>2.014512027082149</v>
       </c>
       <c r="Q5" s="4">
-        <v>1.350496407292254</v>
+        <v>0.1213385858724559</v>
       </c>
       <c r="R5" s="5">
-        <v>569</v>
+        <v>565</v>
       </c>
       <c r="S5" s="5">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -3057,16 +3057,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>-0.1485042415266403</v>
+        <v>-0.1518853318357287</v>
       </c>
       <c r="O3" s="5">
         <v>912</v>
       </c>
       <c r="P3" s="4">
-        <v>0.0859936900615717</v>
+        <v>0.08592723669272113</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.08169180333727909</v>
+        <v>0.0816353789929839</v>
       </c>
       <c r="R3" s="5">
         <v>912</v>
@@ -3116,16 +3116,16 @@
         <v>14</v>
       </c>
       <c r="N4" s="4">
-        <v>0.7205613532272972</v>
+        <v>0.5608419904237962</v>
       </c>
       <c r="O4" s="5">
         <v>681</v>
       </c>
       <c r="P4" s="4">
-        <v>2.676841877700531</v>
+        <v>2.654329847035218</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.1857500547599551</v>
+        <v>0.1168850210615551</v>
       </c>
       <c r="R4" s="5">
         <v>667</v>
@@ -3175,16 +3175,16 @@
         <v>14</v>
       </c>
       <c r="N5" s="4">
-        <v>0.077136963486872</v>
+        <v>-0.1834676199578098</v>
       </c>
       <c r="O5" s="5">
         <v>606</v>
       </c>
       <c r="P5" s="4">
-        <v>1.800543682063408</v>
+        <v>1.725769802539979</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.2718783695871222</v>
+        <v>0.111992245396461</v>
       </c>
       <c r="R5" s="5">
         <v>592</v>
@@ -3357,16 +3357,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>0.1176525444832861</v>
+        <v>0.1264718741076649</v>
       </c>
       <c r="O3" s="5">
         <v>887</v>
       </c>
       <c r="P3" s="4">
-        <v>0.08168149122507344</v>
+        <v>0.08115377302531633</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.05375479000831144</v>
+        <v>0.05300441643033803</v>
       </c>
       <c r="R3" s="5">
         <v>887</v>
@@ -3416,16 +3416,16 @@
         <v>0</v>
       </c>
       <c r="N4" s="4">
-        <v>-0.3042899452663385</v>
+        <v>-0.2932596776663559</v>
       </c>
       <c r="O4" s="5">
         <v>847</v>
       </c>
       <c r="P4" s="4">
-        <v>0.1508198978401864</v>
+        <v>0.1507029997005126</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.1045944061445474</v>
+        <v>0.104176113386205</v>
       </c>
       <c r="R4" s="5">
         <v>847</v>
@@ -3475,16 +3475,16 @@
         <v>16</v>
       </c>
       <c r="N5" s="4">
-        <v>0.04839494755280598</v>
+        <v>0.1250223437255047</v>
       </c>
       <c r="O5" s="5">
         <v>750</v>
       </c>
       <c r="P5" s="4">
-        <v>0.2325846200411077</v>
+        <v>0.2140334009264247</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.1089498809115319</v>
+        <v>0.08396978151730565</v>
       </c>
       <c r="R5" s="5">
         <v>734</v>
@@ -3657,16 +3657,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>-0.1545227498594684</v>
+        <v>-0.1407000459766934</v>
       </c>
       <c r="O3" s="5">
         <v>916</v>
       </c>
       <c r="P3" s="4">
-        <v>0.05840847492469877</v>
+        <v>0.05633076429505413</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.05565388151630912</v>
+        <v>0.05350594934891947</v>
       </c>
       <c r="R3" s="5">
         <v>916</v>
@@ -3716,16 +3716,16 @@
         <v>15</v>
       </c>
       <c r="N4" s="4">
-        <v>-0.06357013484805947</v>
+        <v>-0.1487901580767357</v>
       </c>
       <c r="O4" s="5">
         <v>851</v>
       </c>
       <c r="P4" s="4">
-        <v>0.2472712154168003</v>
+        <v>0.2206887113088101</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.1159985150874442</v>
+        <v>0.08563291161295181</v>
       </c>
       <c r="R4" s="5">
         <v>836</v>
@@ -3775,16 +3775,16 @@
         <v>36</v>
       </c>
       <c r="N5" s="4">
-        <v>-0.3008409244280677</v>
+        <v>-0.3928054411153319</v>
       </c>
       <c r="O5" s="5">
         <v>759</v>
       </c>
       <c r="P5" s="4">
-        <v>0.3708021725290634</v>
+        <v>0.3408171006454039</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.1121574624877428</v>
+        <v>0.07768611547345931</v>
       </c>
       <c r="R5" s="5">
         <v>722</v>
@@ -3957,16 +3957,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>0.1184093683526064</v>
+        <v>0.1308387403005464</v>
       </c>
       <c r="O3" s="5">
         <v>887</v>
       </c>
       <c r="P3" s="4">
-        <v>0.08744806846074012</v>
+        <v>0.08662078134661569</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.06096582809511136</v>
+        <v>0.05981643739666229</v>
       </c>
       <c r="R3" s="5">
         <v>887</v>
@@ -4016,16 +4016,16 @@
         <v>0</v>
       </c>
       <c r="N4" s="4">
-        <v>0.1647925511081258</v>
+        <v>0.1807047515067097</v>
       </c>
       <c r="O4" s="5">
         <v>849</v>
       </c>
       <c r="P4" s="4">
-        <v>0.1499922163048936</v>
+        <v>0.149352369783408</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.1097595923524725</v>
+        <v>0.1087161349346532</v>
       </c>
       <c r="R4" s="5">
         <v>849</v>
@@ -4075,16 +4075,16 @@
         <v>16</v>
       </c>
       <c r="N5" s="4">
-        <v>0.0740795643652709</v>
+        <v>0.1448187072928691</v>
       </c>
       <c r="O5" s="5">
         <v>744</v>
       </c>
       <c r="P5" s="4">
-        <v>0.2399371899440081</v>
+        <v>0.227426330957145</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.1032569483352546</v>
+        <v>0.08428534025551759</v>
       </c>
       <c r="R5" s="5">
         <v>728</v>
@@ -4257,16 +4257,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>-0.02725744240390541</v>
+        <v>-0.02472165172365948</v>
       </c>
       <c r="O3" s="5">
         <v>911</v>
       </c>
       <c r="P3" s="4">
-        <v>0.06610130235708273</v>
+        <v>0.06607552875599029</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.06146928905572296</v>
+        <v>0.06142079459507022</v>
       </c>
       <c r="R3" s="5">
         <v>911</v>
@@ -4316,22 +4316,22 @@
         <v>36</v>
       </c>
       <c r="N4" s="4">
-        <v>0.5504812285231078</v>
+        <v>0.01516088818607386</v>
       </c>
       <c r="O4" s="5">
         <v>759</v>
       </c>
       <c r="P4" s="4">
-        <v>1.81912977691015</v>
+        <v>1.571480901248874</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.5475778540501073</v>
+        <v>0.1560697713158139</v>
       </c>
       <c r="R4" s="5">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="S4" s="5">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="25" customHeight="1">
@@ -4375,16 +4375,16 @@
         <v>33</v>
       </c>
       <c r="N5" s="4">
-        <v>0.4316319560934572</v>
+        <v>-0.1147621056552346</v>
       </c>
       <c r="O5" s="5">
         <v>667</v>
       </c>
       <c r="P5" s="4">
-        <v>1.62390255172819</v>
+        <v>1.366863113548165</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.5573806862063017</v>
+        <v>0.1537424667505171</v>
       </c>
       <c r="R5" s="5">
         <v>634</v>
@@ -4521,13 +4521,13 @@
         <v>1.636225266362253</v>
       </c>
       <c r="H3" s="4">
-        <v>1.603839398119619</v>
+        <v>1.570380141415235</v>
       </c>
       <c r="I3" s="4">
-        <v>0.2503887752842477</v>
+        <v>0.1738998457870957</v>
       </c>
       <c r="J3" s="4">
-        <v>2.460112327675686</v>
+        <v>2.447410665269545</v>
       </c>
       <c r="K3" s="4">
         <v>85.1932485322896</v>
@@ -4571,13 +4571,13 @@
         <v>0.684931506849315</v>
       </c>
       <c r="H4" s="4">
-        <v>0.3729118252549304</v>
+        <v>0.3703771990548365</v>
       </c>
       <c r="I4" s="4">
-        <v>0.3080361107466925</v>
+        <v>0.3052688648751573</v>
       </c>
       <c r="J4" s="4">
-        <v>0.3790126744400553</v>
+        <v>0.3805173488212104</v>
       </c>
       <c r="K4" s="4">
         <v>81.84100580871623</v>
@@ -4603,13 +4603,13 @@
         <v>19</v>
       </c>
       <c r="B5" s="3">
-        <v>89.15525114155251</v>
+        <v>88.58447488584474</v>
       </c>
       <c r="C5" s="3">
         <v>2.777777777777778</v>
       </c>
       <c r="D5" s="3">
-        <v>8.06697108066971</v>
+        <v>8.637747336377473</v>
       </c>
       <c r="E5" s="3">
         <v>1.36986301369863</v>
@@ -4618,16 +4618,16 @@
         <v>3.006088280060883</v>
       </c>
       <c r="G5" s="3">
-        <v>3.691019786910198</v>
+        <v>4.26179604261796</v>
       </c>
       <c r="H5" s="4">
-        <v>0.8869655227861335</v>
+        <v>0.7437813700135029</v>
       </c>
       <c r="I5" s="4">
-        <v>0.3572363640778014</v>
+        <v>0.1490043552807545</v>
       </c>
       <c r="J5" s="4">
-        <v>1.368039205131769</v>
+        <v>1.244933821992914</v>
       </c>
       <c r="K5" s="4">
         <v>91.19033381998136</v>
@@ -4653,13 +4653,13 @@
         <v>20</v>
       </c>
       <c r="B6" s="3">
-        <v>83.67579908675799</v>
+        <v>83.29528158295282</v>
       </c>
       <c r="C6" s="3">
         <v>8.181126331811264</v>
       </c>
       <c r="D6" s="3">
-        <v>8.143074581430746</v>
+        <v>8.52359208523592</v>
       </c>
       <c r="E6" s="3">
         <v>1.06544901065449</v>
@@ -4668,16 +4668,16 @@
         <v>4.794520547945205</v>
       </c>
       <c r="G6" s="3">
-        <v>2.28310502283105</v>
+        <v>2.663622526636225</v>
       </c>
       <c r="H6" s="4">
-        <v>0.6259276687395378</v>
+        <v>0.5975964861841845</v>
       </c>
       <c r="I6" s="4">
-        <v>0.3137198006770681</v>
+        <v>0.2542091695958678</v>
       </c>
       <c r="J6" s="4">
-        <v>0.8256905300766807</v>
+        <v>0.8233796654456426</v>
       </c>
       <c r="K6" s="4">
         <v>82.97303243976449</v>
@@ -4721,13 +4721,13 @@
         <v>3.729071537290715</v>
       </c>
       <c r="H7" s="4">
-        <v>1.925092631974459</v>
+        <v>1.715791064716045</v>
       </c>
       <c r="I7" s="4">
-        <v>0.4152786041209838</v>
+        <v>0.06994071716058758</v>
       </c>
       <c r="J7" s="4">
-        <v>2.506180676103521</v>
+        <v>2.30726718224309</v>
       </c>
       <c r="K7" s="4">
         <v>91.44940929187509</v>
@@ -4753,13 +4753,13 @@
         <v>22</v>
       </c>
       <c r="B8" s="3">
-        <v>83.0289193302892</v>
+        <v>82.87671232876713</v>
       </c>
       <c r="C8" s="3">
         <v>4.680365296803653</v>
       </c>
       <c r="D8" s="3">
-        <v>12.29071537290715</v>
+        <v>12.44292237442922</v>
       </c>
       <c r="E8" s="3">
         <v>1.560121765601218</v>
@@ -4768,16 +4768,16 @@
         <v>7.229832572298325</v>
       </c>
       <c r="G8" s="3">
-        <v>3.50076103500761</v>
+        <v>3.65296803652968</v>
       </c>
       <c r="H8" s="4">
-        <v>1.022242104555708</v>
+        <v>0.959941866643149</v>
       </c>
       <c r="I8" s="4">
-        <v>0.2498225050975524</v>
+        <v>0.1302459304243615</v>
       </c>
       <c r="J8" s="4">
-        <v>1.558108618327527</v>
+        <v>1.51445923782565</v>
       </c>
       <c r="K8" s="4">
         <v>88.70869961378773</v>
@@ -4803,13 +4803,13 @@
         <v>23</v>
       </c>
       <c r="B9" s="3">
-        <v>75.98934550989345</v>
+        <v>75.79908675799086</v>
       </c>
       <c r="C9" s="3">
         <v>12.13850837138508</v>
       </c>
       <c r="D9" s="3">
-        <v>11.87214611872146</v>
+        <v>12.06240487062405</v>
       </c>
       <c r="E9" s="3">
         <v>0.76103500761035</v>
@@ -4818,16 +4818,16 @@
         <v>7.686453576864535</v>
       </c>
       <c r="G9" s="3">
-        <v>3.424657534246575</v>
+        <v>3.614916286149163</v>
       </c>
       <c r="H9" s="4">
-        <v>0.6400165041591689</v>
+        <v>0.617156099704221</v>
       </c>
       <c r="I9" s="4">
-        <v>0.364640460960513</v>
+        <v>0.299447326861645</v>
       </c>
       <c r="J9" s="4">
-        <v>0.7400597039316763</v>
+        <v>0.7556767799517426</v>
       </c>
       <c r="K9" s="4">
         <v>80.37694529866741</v>
@@ -4871,13 +4871,13 @@
         <v>0.2663622526636225</v>
       </c>
       <c r="H10" s="4">
-        <v>0.1850277775921205</v>
+        <v>0.1799381467357229</v>
       </c>
       <c r="I10" s="4">
-        <v>0.1405527223346537</v>
+        <v>0.1345444813789973</v>
       </c>
       <c r="J10" s="4">
-        <v>0.1806834117579051</v>
+        <v>0.1726927653694533</v>
       </c>
       <c r="K10" s="4">
         <v>88.48489319624339</v>
@@ -4903,13 +4903,13 @@
         <v>25</v>
       </c>
       <c r="B11" s="3">
-        <v>80.28919330289193</v>
+        <v>80.25114155251141</v>
       </c>
       <c r="C11" s="3">
         <v>5.32724505327245</v>
       </c>
       <c r="D11" s="3">
-        <v>14.38356164383562</v>
+        <v>14.42161339421613</v>
       </c>
       <c r="E11" s="3">
         <v>5.098934550989346</v>
@@ -4918,16 +4918,16 @@
         <v>7.30593607305936</v>
       </c>
       <c r="G11" s="3">
-        <v>1.97869101978691</v>
+        <v>2.016742770167427</v>
       </c>
       <c r="H11" s="4">
-        <v>2.344289930510119</v>
+        <v>2.247611578097039</v>
       </c>
       <c r="I11" s="4">
-        <v>0.4421771765360566</v>
+        <v>0.247134449548202</v>
       </c>
       <c r="J11" s="4">
-        <v>3.110305103910154</v>
+        <v>3.041657501243095</v>
       </c>
       <c r="K11" s="4">
         <v>85.45979198376453</v>
@@ -4953,13 +4953,13 @@
         <v>26</v>
       </c>
       <c r="B12" s="3">
-        <v>81.46879756468797</v>
+        <v>80.97412480974124</v>
       </c>
       <c r="C12" s="3">
         <v>5.93607305936073</v>
       </c>
       <c r="D12" s="3">
-        <v>12.5951293759513</v>
+        <v>13.08980213089802</v>
       </c>
       <c r="E12" s="3">
         <v>2.43531202435312</v>
@@ -4968,16 +4968,16 @@
         <v>2.815829528158295</v>
       </c>
       <c r="G12" s="3">
-        <v>7.343987823439877</v>
+        <v>7.838660578386605</v>
       </c>
       <c r="H12" s="4">
-        <v>1.838488695398447</v>
+        <v>1.388219601380314</v>
       </c>
       <c r="I12" s="4">
-        <v>0.8358756961060667</v>
+        <v>0.1113536696390186</v>
       </c>
       <c r="J12" s="4">
-        <v>2.125875047597869</v>
+        <v>1.695478875133292</v>
       </c>
       <c r="K12" s="4">
         <v>89.91816285113737</v>
@@ -5021,13 +5021,13 @@
         <v>1.06544901065449</v>
       </c>
       <c r="H13" s="4">
-        <v>1.49352178180399</v>
+        <v>1.462858866921197</v>
       </c>
       <c r="I13" s="4">
-        <v>0.1655228954233371</v>
+        <v>0.1007430603244419</v>
       </c>
       <c r="J13" s="4">
-        <v>2.305471194077953</v>
+        <v>2.289060927146529</v>
       </c>
       <c r="K13" s="4">
         <v>88.72610764244811</v>
@@ -5071,13 +5071,13 @@
         <v>0.60882800608828</v>
       </c>
       <c r="H14" s="4">
-        <v>0.1515712648897049</v>
+        <v>0.1456416720987737</v>
       </c>
       <c r="I14" s="4">
-        <v>0.08761797946955768</v>
+        <v>0.07977548826804207</v>
       </c>
       <c r="J14" s="4">
-        <v>0.1251559532766653</v>
+        <v>0.1162443263743348</v>
       </c>
       <c r="K14" s="4">
         <v>87.85992555317405</v>
@@ -5121,13 +5121,13 @@
         <v>1.97869101978691</v>
       </c>
       <c r="H15" s="4">
-        <v>0.2186324227647951</v>
+        <v>0.1996475856247218</v>
       </c>
       <c r="I15" s="4">
-        <v>0.09253492400897043</v>
+        <v>0.07141873043002246</v>
       </c>
       <c r="J15" s="4">
-        <v>0.3241583307291821</v>
+        <v>0.3084494461719705</v>
       </c>
       <c r="K15" s="4">
         <v>95.73600368610154</v>
@@ -5171,13 +5171,13 @@
         <v>0.60882800608828</v>
       </c>
       <c r="H16" s="4">
-        <v>0.1555847253037042</v>
+        <v>0.1512289215899046</v>
       </c>
       <c r="I16" s="4">
-        <v>0.09027339359402527</v>
+        <v>0.08389484831021789</v>
       </c>
       <c r="J16" s="4">
-        <v>0.1272706127858137</v>
+        <v>0.1194679839781412</v>
       </c>
       <c r="K16" s="4">
         <v>88.05642272129553</v>
@@ -5203,13 +5203,13 @@
         <v>31</v>
       </c>
       <c r="B17" s="3">
-        <v>86.37747336377474</v>
+        <v>86.3013698630137</v>
       </c>
       <c r="C17" s="3">
         <v>3.691019786910198</v>
       </c>
       <c r="D17" s="3">
-        <v>9.931506849315069</v>
+        <v>10.0076103500761</v>
       </c>
       <c r="E17" s="3">
         <v>3.50076103500761</v>
@@ -5218,16 +5218,16 @@
         <v>3.881278538812785</v>
       </c>
       <c r="G17" s="3">
-        <v>2.549467275494673</v>
+        <v>2.625570776255707</v>
       </c>
       <c r="H17" s="4">
-        <v>1.140742792946026</v>
+        <v>0.9775532175490731</v>
       </c>
       <c r="I17" s="4">
-        <v>0.3552298773440029</v>
+        <v>0.117401019601971</v>
       </c>
       <c r="J17" s="4">
-        <v>1.996634691105638</v>
+        <v>1.855998717436995</v>
       </c>
       <c r="K17" s="4">
         <v>91.66644663953859</v>
@@ -6198,13 +6198,13 @@
         <v>19</v>
       </c>
       <c r="B5" s="5">
-        <v>2343</v>
+        <v>2328</v>
       </c>
       <c r="C5" s="5">
         <v>73</v>
       </c>
       <c r="D5" s="5">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="E5" s="5">
         <v>36</v>
@@ -6213,7 +6213,7 @@
         <v>79</v>
       </c>
       <c r="G5" s="5">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="H5" s="5">
         <v>36</v>
@@ -6242,13 +6242,13 @@
         <v>20</v>
       </c>
       <c r="B6" s="5">
-        <v>2199</v>
+        <v>2189</v>
       </c>
       <c r="C6" s="5">
         <v>215</v>
       </c>
       <c r="D6" s="5">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="E6" s="5">
         <v>28</v>
@@ -6257,7 +6257,7 @@
         <v>126</v>
       </c>
       <c r="G6" s="5">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="H6" s="5">
         <v>28</v>
@@ -6330,13 +6330,13 @@
         <v>22</v>
       </c>
       <c r="B8" s="5">
-        <v>2182</v>
+        <v>2178</v>
       </c>
       <c r="C8" s="5">
         <v>123</v>
       </c>
       <c r="D8" s="5">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="E8" s="5">
         <v>41</v>
@@ -6345,7 +6345,7 @@
         <v>190</v>
       </c>
       <c r="G8" s="5">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H8" s="5">
         <v>41</v>
@@ -6374,13 +6374,13 @@
         <v>23</v>
       </c>
       <c r="B9" s="5">
-        <v>1997</v>
+        <v>1992</v>
       </c>
       <c r="C9" s="5">
         <v>319</v>
       </c>
       <c r="D9" s="5">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="E9" s="5">
         <v>20</v>
@@ -6389,7 +6389,7 @@
         <v>202</v>
       </c>
       <c r="G9" s="5">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="H9" s="5">
         <v>20</v>
@@ -6462,13 +6462,13 @@
         <v>25</v>
       </c>
       <c r="B11" s="5">
-        <v>2110</v>
+        <v>2109</v>
       </c>
       <c r="C11" s="5">
         <v>140</v>
       </c>
       <c r="D11" s="5">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E11" s="5">
         <v>134</v>
@@ -6477,7 +6477,7 @@
         <v>192</v>
       </c>
       <c r="G11" s="5">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="H11" s="5">
         <v>134</v>
@@ -6506,13 +6506,13 @@
         <v>26</v>
       </c>
       <c r="B12" s="5">
-        <v>2141</v>
+        <v>2128</v>
       </c>
       <c r="C12" s="5">
         <v>156</v>
       </c>
       <c r="D12" s="5">
-        <v>331</v>
+        <v>344</v>
       </c>
       <c r="E12" s="5">
         <v>64</v>
@@ -6521,7 +6521,7 @@
         <v>74</v>
       </c>
       <c r="G12" s="5">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="H12" s="5">
         <v>64</v>
@@ -6726,13 +6726,13 @@
         <v>31</v>
       </c>
       <c r="B17" s="5">
-        <v>2270</v>
+        <v>2268</v>
       </c>
       <c r="C17" s="5">
         <v>97</v>
       </c>
       <c r="D17" s="5">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="E17" s="5">
         <v>92</v>
@@ -6741,7 +6741,7 @@
         <v>102</v>
       </c>
       <c r="G17" s="5">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H17" s="5">
         <v>92</v>
@@ -6924,16 +6924,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>-0.07952600696503768</v>
+        <v>-0.08263790664204862</v>
       </c>
       <c r="O3" s="5">
         <v>902</v>
       </c>
       <c r="P3" s="4">
-        <v>0.127594317313434</v>
+        <v>0.1274856544510622</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.1197876135305364</v>
+        <v>0.1197483889405126</v>
       </c>
       <c r="R3" s="5">
         <v>902</v>
@@ -6983,16 +6983,16 @@
         <v>20</v>
       </c>
       <c r="N4" s="4">
-        <v>0.6940438841340045</v>
+        <v>0.498393211120856</v>
       </c>
       <c r="O4" s="5">
         <v>682</v>
       </c>
       <c r="P4" s="4">
-        <v>2.595194324235674</v>
+        <v>2.594494033635464</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.2929372889088343</v>
+        <v>0.2429121498085089</v>
       </c>
       <c r="R4" s="5">
         <v>662</v>
@@ -7042,16 +7042,16 @@
         <v>23</v>
       </c>
       <c r="N5" s="4">
-        <v>0.4807830131816727</v>
+        <v>0.08709197228927223</v>
       </c>
       <c r="O5" s="5">
         <v>580</v>
       </c>
       <c r="P5" s="4">
-        <v>2.201858260601917</v>
+        <v>2.093931482582467</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.4113136081071763</v>
+        <v>0.1795703463498288</v>
       </c>
       <c r="R5" s="5">
         <v>557</v>
@@ -7224,16 +7224,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>-0.1418326304085579</v>
+        <v>-0.1144404631704674</v>
       </c>
       <c r="O3" s="5">
         <v>818</v>
       </c>
       <c r="P3" s="4">
-        <v>0.2116049344070962</v>
+        <v>0.2099520676202802</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.2066701186441467</v>
+        <v>0.2052993056822798</v>
       </c>
       <c r="R3" s="5">
         <v>818</v>
@@ -7283,16 +7283,16 @@
         <v>14</v>
       </c>
       <c r="N4" s="4">
-        <v>0.5441005212699151</v>
+        <v>0.4458276023215149</v>
       </c>
       <c r="O4" s="5">
         <v>770</v>
       </c>
       <c r="P4" s="4">
-        <v>0.4778455021642342</v>
+        <v>0.4721126721674659</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.4313050510100551</v>
+        <v>0.425048530525124</v>
       </c>
       <c r="R4" s="5">
         <v>767</v>
@@ -7342,16 +7342,16 @@
         <v>15</v>
       </c>
       <c r="N5" s="4">
-        <v>0.2899082436118227</v>
+        <v>0.2897520276892465</v>
       </c>
       <c r="O5" s="5">
         <v>569</v>
       </c>
       <c r="P5" s="4">
-        <v>0.4420030558687104</v>
+        <v>0.4419914556764398</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.2870435193349296</v>
+        <v>0.2870452112041272</v>
       </c>
       <c r="R5" s="5">
         <v>554</v>
@@ -7524,16 +7524,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>-0.01665483512680748</v>
+        <v>-0.01644762598698435</v>
       </c>
       <c r="O3" s="5">
         <v>906</v>
       </c>
       <c r="P3" s="4">
-        <v>0.0874347811056862</v>
+        <v>0.08743693420979438</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.08143020088285033</v>
+        <v>0.08142943069376708</v>
       </c>
       <c r="R3" s="5">
         <v>906</v>
@@ -7583,22 +7583,22 @@
         <v>76</v>
       </c>
       <c r="N4" s="4">
-        <v>1.293570856884371</v>
+        <v>0.5426721083422308</v>
       </c>
       <c r="O4" s="5">
         <v>791</v>
       </c>
       <c r="P4" s="4">
-        <v>1.975888766367197</v>
+        <v>1.627182890673548</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.7726321898742268</v>
+        <v>0.2109452044122176</v>
       </c>
       <c r="R4" s="5">
-        <v>739</v>
+        <v>727</v>
       </c>
       <c r="S4" s="5">
-        <v>52</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="25" customHeight="1">
@@ -7642,22 +7642,22 @@
         <v>44</v>
       </c>
       <c r="N5" s="4">
-        <v>0.1360325530645945</v>
+        <v>-0.07426859917904949</v>
       </c>
       <c r="O5" s="5">
         <v>743</v>
       </c>
       <c r="P5" s="4">
-        <v>0.6007731230582685</v>
+        <v>0.5204567834301084</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.2754353162140007</v>
+        <v>0.1723020306149082</v>
       </c>
       <c r="R5" s="5">
-        <v>698</v>
+        <v>695</v>
       </c>
       <c r="S5" s="5">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -7824,16 +7824,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>-0.1367307879189856</v>
+        <v>-0.1441291445389652</v>
       </c>
       <c r="O3" s="5">
         <v>880</v>
       </c>
       <c r="P3" s="4">
-        <v>0.1709549019958447</v>
+        <v>0.1707180316623776</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.1620522584643504</v>
+        <v>0.16194565990005</v>
       </c>
       <c r="R3" s="5">
         <v>880</v>
@@ -7883,22 +7883,22 @@
         <v>62</v>
       </c>
       <c r="N4" s="4">
-        <v>1.283885810032353</v>
+        <v>0.8904624545029947</v>
       </c>
       <c r="O4" s="5">
         <v>743</v>
       </c>
       <c r="P4" s="4">
-        <v>1.143460215702502</v>
+        <v>1.067217933611422</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.5043890735198354</v>
+        <v>0.348717818701791</v>
       </c>
       <c r="R4" s="5">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="S4" s="5">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="25" customHeight="1">
@@ -7942,22 +7942,22 @@
         <v>26</v>
       </c>
       <c r="N5" s="4">
-        <v>0.2010141678128688</v>
+        <v>0.08526686773438996</v>
       </c>
       <c r="O5" s="5">
         <v>636</v>
       </c>
       <c r="P5" s="4">
-        <v>0.5759316171720582</v>
+        <v>0.5683197223094213</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.3134095690984464</v>
+        <v>0.279127093419739</v>
       </c>
       <c r="R5" s="5">
-        <v>618</v>
+        <v>611</v>
       </c>
       <c r="S5" s="5">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -8124,16 +8124,16 @@
         <v>0</v>
       </c>
       <c r="N3" s="4">
-        <v>0.02264211352126358</v>
+        <v>0.02479095247690566</v>
       </c>
       <c r="O3" s="5">
         <v>916</v>
       </c>
       <c r="P3" s="4">
-        <v>0.0523291474879299</v>
+        <v>0.05230599647870583</v>
       </c>
       <c r="Q3" s="4">
-        <v>0.04705361015301595</v>
+        <v>0.04701375987109432</v>
       </c>
       <c r="R3" s="5">
         <v>916</v>
@@ -8183,16 +8183,16 @@
         <v>46</v>
       </c>
       <c r="N4" s="4">
-        <v>1.069910084373121</v>
+        <v>0.5042543234449113</v>
       </c>
       <c r="O4" s="5">
         <v>736</v>
       </c>
       <c r="P4" s="4">
-        <v>2.990761237546193</v>
+        <v>2.741317256982992</v>
       </c>
       <c r="Q4" s="4">
-        <v>0.5648908010719612</v>
+        <v>0.1015787760957775</v>
       </c>
       <c r="R4" s="5">
         <v>692</v>
@@ -8242,16 +8242,16 @@
         <v>54</v>
       </c>
       <c r="N5" s="4">
-        <v>0.7856910444720416</v>
+        <v>-0.02196266653481871</v>
       </c>
       <c r="O5" s="5">
         <v>652</v>
       </c>
       <c r="P5" s="4">
-        <v>2.895896697993588</v>
+        <v>2.490860085213113</v>
       </c>
       <c r="Q5" s="4">
-        <v>0.8061857181420243</v>
+        <v>0.06844833604691607</v>
       </c>
       <c r="R5" s="5">
         <v>598</v>

</xml_diff>